<commit_message>
Content: 문구 엑셀에 '홈' 시트 추가 — 시안 C 홈(index-c.html) 46 줄, 생성기 copy_home.py
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/content-export/04_사업영역_문구.xlsx
+++ b/content-export/04_사업영역_문구.xlsx
@@ -8,16 +8,18 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="안내" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="스마트 제조" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="에너지 인프라" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="인공지능 플랫폼" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="화합물 전력 반도체" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="홈" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="스마트 제조" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="에너지 인프라" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="인공지능 플랫폼" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="화합물 전력 반도체" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'스마트 제조'!$A$1:$J$141</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'에너지 인프라'!$A$1:$J$189</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'인공지능 플랫폼'!$A$1:$J$47</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'화합물 전력 반도체'!$A$1:$J$25</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'홈'!$A$1:$J$47</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'스마트 제조'!$A$1:$J$141</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'에너지 인프라'!$A$1:$J$189</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'인공지능 플랫폼'!$A$1:$J$47</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'화합물 전력 반도체'!$A$1:$J$25</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -500,7 +502,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B29"/>
+  <dimension ref="B1:B34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -686,12 +688,1822 @@
         </is>
       </c>
     </row>
+    <row r="30">
+      <c r="B30" s="3" t="inlineStr">
+        <is>
+          <t>홈 시트 (2026-10-07 추가)</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="B31" s="2" t="inlineStr">
+        <is>
+          <t>홈(시안 C, index-c.html)의 문구입니다. 히어로 · Business · Who we are · News 순서로, 화면에 보이는 순서대로 담았습니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="B32" s="2" t="inlineStr">
+        <is>
+          <t>채우는 법은 사업영역 시트와 같습니다 — 노란 칸에 한글, 파란 칸에 영문. 같은 문구가 여러 자리에 있으면(사업영역 이름이 히어로 탭 · 카드에 함께 있는 것 등) 한 줄로 합쳤습니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="B33" s="2" t="inlineStr">
+        <is>
+          <t>보도자료 기사 제목 · 날짜는 게시판 글이라 넣지 않았습니다. 게시판에서 고칩니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="B34" s="2" t="inlineStr">
+        <is>
+          <t>사업영역 시트는 A-1 장 기준으로 뽑은 그대로입니다(2026-09-17). 홈 시트만 지금 시안 C 기준입니다.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J47"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="6" customWidth="1" min="1" max="1"/>
+    <col width="24" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="8" customWidth="1" min="4" max="4"/>
+    <col width="6" customWidth="1" min="5" max="5"/>
+    <col width="54" customWidth="1" min="6" max="6"/>
+    <col width="54" customWidth="1" min="7" max="7"/>
+    <col width="54" customWidth="1" min="8" max="8"/>
+    <col width="20" customWidth="1" min="9" max="9"/>
+    <col width="44" customWidth="1" min="10" max="10"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="24" customHeight="1">
+      <c r="A1" s="4" t="inlineStr">
+        <is>
+          <t>순번</t>
+        </is>
+      </c>
+      <c r="B1" s="4" t="inlineStr">
+        <is>
+          <t>섹션</t>
+        </is>
+      </c>
+      <c r="C1" s="4" t="inlineStr">
+        <is>
+          <t>자리</t>
+        </is>
+      </c>
+      <c r="D1" s="4" t="inlineStr">
+        <is>
+          <t>구분</t>
+        </is>
+      </c>
+      <c r="E1" s="4" t="inlineStr">
+        <is>
+          <t>묶음</t>
+        </is>
+      </c>
+      <c r="F1" s="4" t="inlineStr">
+        <is>
+          <t>현재 문구</t>
+        </is>
+      </c>
+      <c r="G1" s="4" t="inlineStr">
+        <is>
+          <t>변경 문구</t>
+        </is>
+      </c>
+      <c r="H1" s="4" t="inlineStr">
+        <is>
+          <t>영문 문구</t>
+        </is>
+      </c>
+      <c r="I1" s="4" t="inlineStr">
+        <is>
+          <t>비고</t>
+        </is>
+      </c>
+      <c r="J1" s="4" t="inlineStr">
+        <is>
+          <t>자리표(건드리지 마세요)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="5" t="inlineStr">
+        <is>
+          <t>히어로</t>
+        </is>
+      </c>
+      <c r="C2" s="5" t="inlineStr">
+        <is>
+          <t>페이지 제목(화면 낭독기용)</t>
+        </is>
+      </c>
+      <c r="D2" s="5" t="inlineStr">
+        <is>
+          <t>숨김글</t>
+        </is>
+      </c>
+      <c r="E2" s="5" t="n"/>
+      <c r="F2" s="6" t="inlineStr">
+        <is>
+          <t>에이프로 APRO</t>
+        </is>
+      </c>
+      <c r="G2" s="7" t="n"/>
+      <c r="H2" s="8" t="n"/>
+      <c r="I2" s="5" t="n"/>
+      <c r="J2" s="9" t="inlineStr">
+        <is>
+          <t>/html/body/div[3]/h1|text</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="5" t="inlineStr">
+        <is>
+          <t>히어로</t>
+        </is>
+      </c>
+      <c r="C3" s="5" t="inlineStr">
+        <is>
+          <t>메인 문구</t>
+        </is>
+      </c>
+      <c r="D3" s="5" t="inlineStr">
+        <is>
+          <t>문구</t>
+        </is>
+      </c>
+      <c r="E3" s="5" t="n"/>
+      <c r="F3" s="6" t="inlineStr">
+        <is>
+          <t>에이프로는 함께 나아가는 기업입니다</t>
+        </is>
+      </c>
+      <c r="G3" s="7" t="n"/>
+      <c r="H3" s="8" t="n"/>
+      <c r="I3" s="5" t="n"/>
+      <c r="J3" s="9" t="inlineStr">
+        <is>
+          <t>/html/body/div[3]/section[1]/div/div/div[1]/p[1]|text</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>히어로</t>
+        </is>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>서브 문구</t>
+        </is>
+      </c>
+      <c r="D4" s="5" t="inlineStr">
+        <is>
+          <t>문구</t>
+        </is>
+      </c>
+      <c r="E4" s="5" t="n"/>
+      <c r="F4" s="6" t="inlineStr">
+        <is>
+          <t>당신이 향하는 세상으로 우리도 같이 나아갑니다</t>
+        </is>
+      </c>
+      <c r="G4" s="7" t="n"/>
+      <c r="H4" s="8" t="n"/>
+      <c r="I4" s="5" t="n"/>
+      <c r="J4" s="9" t="inlineStr">
+        <is>
+          <t>/html/body/div[3]/section[1]/div/div/div[1]/p[2]|text</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>히어로</t>
+        </is>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>하단 탭</t>
+        </is>
+      </c>
+      <c r="D5" s="5" t="inlineStr">
+        <is>
+          <t>문구</t>
+        </is>
+      </c>
+      <c r="E5" s="5" t="n"/>
+      <c r="F5" s="6" t="inlineStr">
+        <is>
+          <t>에이프로</t>
+        </is>
+      </c>
+      <c r="G5" s="7" t="n"/>
+      <c r="H5" s="8" t="n"/>
+      <c r="I5" s="5" t="n"/>
+      <c r="J5" s="9" t="inlineStr">
+        <is>
+          <t>/html/body/div[3]/section[1]/div/div/div[2]/div/div/span[1]/span|text</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>히어로 · Business</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>하단 탭 · 카드 이름</t>
+        </is>
+      </c>
+      <c r="D6" s="5" t="inlineStr">
+        <is>
+          <t>문구</t>
+        </is>
+      </c>
+      <c r="E6" s="5" t="n"/>
+      <c r="F6" s="6" t="inlineStr">
+        <is>
+          <t>스마트 제조</t>
+        </is>
+      </c>
+      <c r="G6" s="7" t="n"/>
+      <c r="H6" s="8" t="n"/>
+      <c r="I6" s="5" t="inlineStr">
+        <is>
+          <t>같은 문구 3 곳 — 한 줄로 합침
+카드 제목 자리는 두 줄로 나눠 보입니다 — 줄 나눌 곳이 따로 있으면 비고에 적어 주세요
+GNB · 메가 메뉴 · 푸터의 사업영역 이름도 함께 고칩니다</t>
+        </is>
+      </c>
+      <c r="J6" s="9" t="inlineStr">
+        <is>
+          <t>/html/body/div[3]/section[1]/div/div/div[2]/div/div/span[2]/span|text
+/html/body/div[3]/section[2]/div[2]/ul/li[1]/span/span|text
+/html/body/div[3]/section[2]/div[2]/ul/li[1]/div/div[1]/div/h3/a|text</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>히어로 · Business</t>
+        </is>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>하단 탭 · 카드 이름</t>
+        </is>
+      </c>
+      <c r="D7" s="5" t="inlineStr">
+        <is>
+          <t>문구</t>
+        </is>
+      </c>
+      <c r="E7" s="5" t="n"/>
+      <c r="F7" s="6" t="inlineStr">
+        <is>
+          <t>에너지 인프라</t>
+        </is>
+      </c>
+      <c r="G7" s="7" t="n"/>
+      <c r="H7" s="8" t="n"/>
+      <c r="I7" s="5" t="inlineStr">
+        <is>
+          <t>같은 문구 3 곳 — 한 줄로 합침
+카드 제목 자리는 두 줄로 나눠 보입니다 — 줄 나눌 곳이 따로 있으면 비고에 적어 주세요
+GNB · 메가 메뉴 · 푸터의 사업영역 이름도 함께 고칩니다</t>
+        </is>
+      </c>
+      <c r="J7" s="9" t="inlineStr">
+        <is>
+          <t>/html/body/div[3]/section[1]/div/div/div[2]/div/div/span[3]/span|text
+/html/body/div[3]/section[2]/div[2]/ul/li[2]/span/span|text
+/html/body/div[3]/section[2]/div[2]/ul/li[2]/div/div[1]/div/h3/a|text</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>히어로 · Business</t>
+        </is>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>하단 탭 · 카드 이름</t>
+        </is>
+      </c>
+      <c r="D8" s="5" t="inlineStr">
+        <is>
+          <t>문구</t>
+        </is>
+      </c>
+      <c r="E8" s="5" t="n"/>
+      <c r="F8" s="6" t="inlineStr">
+        <is>
+          <t>인공지능 플랫폼</t>
+        </is>
+      </c>
+      <c r="G8" s="7" t="n"/>
+      <c r="H8" s="8" t="n"/>
+      <c r="I8" s="5" t="inlineStr">
+        <is>
+          <t>같은 문구 3 곳 — 한 줄로 합침
+카드 제목 자리는 두 줄로 나눠 보입니다 — 줄 나눌 곳이 따로 있으면 비고에 적어 주세요
+GNB · 메가 메뉴 · 푸터의 사업영역 이름도 함께 고칩니다</t>
+        </is>
+      </c>
+      <c r="J8" s="9" t="inlineStr">
+        <is>
+          <t>/html/body/div[3]/section[1]/div/div/div[2]/div/div/span[4]/span|text
+/html/body/div[3]/section[2]/div[2]/ul/li[3]/span/span|text
+/html/body/div[3]/section[2]/div[2]/ul/li[3]/div/div[1]/div/h3/a|text</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>히어로 · Business</t>
+        </is>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>하단 탭 · 카드 이름</t>
+        </is>
+      </c>
+      <c r="D9" s="5" t="inlineStr">
+        <is>
+          <t>문구</t>
+        </is>
+      </c>
+      <c r="E9" s="5" t="n"/>
+      <c r="F9" s="6" t="inlineStr">
+        <is>
+          <t>화합물 전력 반도체</t>
+        </is>
+      </c>
+      <c r="G9" s="7" t="n"/>
+      <c r="H9" s="8" t="n"/>
+      <c r="I9" s="5" t="inlineStr">
+        <is>
+          <t>같은 문구 3 곳 — 한 줄로 합침
+카드 제목 자리는 두 줄로 나눠 보입니다 — 줄 나눌 곳이 따로 있으면 비고에 적어 주세요
+GNB · 메가 메뉴 · 푸터의 사업영역 이름도 함께 고칩니다</t>
+        </is>
+      </c>
+      <c r="J9" s="9" t="inlineStr">
+        <is>
+          <t>/html/body/div[3]/section[1]/div/div/div[2]/div/div/span[5]/span|text
+/html/body/div[3]/section[2]/div[2]/ul/li[4]/span/span|text
+/html/body/div[3]/section[2]/div[2]/ul/li[4]/div/div[1]/div/h3/a|text</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>Business</t>
+        </is>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>섹션 제목</t>
+        </is>
+      </c>
+      <c r="D10" s="5" t="inlineStr">
+        <is>
+          <t>문구</t>
+        </is>
+      </c>
+      <c r="E10" s="5" t="n"/>
+      <c r="F10" s="6" t="inlineStr">
+        <is>
+          <t>Business</t>
+        </is>
+      </c>
+      <c r="G10" s="7" t="n"/>
+      <c r="H10" s="8" t="inlineStr">
+        <is>
+          <t>Business</t>
+        </is>
+      </c>
+      <c r="I10" s="5" t="n"/>
+      <c r="J10" s="9" t="inlineStr">
+        <is>
+          <t>/html/body/div[3]/section[2]/div[1]/h2|text</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" s="5" t="inlineStr">
+        <is>
+          <t>Business</t>
+        </is>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>섹션 라벨</t>
+        </is>
+      </c>
+      <c r="D11" s="5" t="inlineStr">
+        <is>
+          <t>문구</t>
+        </is>
+      </c>
+      <c r="E11" s="5" t="n"/>
+      <c r="F11" s="6" t="inlineStr">
+        <is>
+          <t>사업영역</t>
+        </is>
+      </c>
+      <c r="G11" s="7" t="n"/>
+      <c r="H11" s="8" t="n"/>
+      <c r="I11" s="5" t="n"/>
+      <c r="J11" s="9" t="inlineStr">
+        <is>
+          <t>/html/body/div[3]/section[2]/div[1]/h2/span|text</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <t>Business · 스마트 제조</t>
+        </is>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>카드 설명</t>
+        </is>
+      </c>
+      <c r="D12" s="5" t="inlineStr">
+        <is>
+          <t>문구</t>
+        </is>
+      </c>
+      <c r="E12" s="5" t="n"/>
+      <c r="F12" s="6" t="inlineStr">
+        <is>
+          <t>이차전지 활성화 공정의 주요 설비를 자체 기술로 만듭니다.
+셀의 성능과 품질을 결정짓는 마지막 공정까지, A-PRO가 책임집니다.</t>
+        </is>
+      </c>
+      <c r="G12" s="7" t="n"/>
+      <c r="H12" s="8" t="n"/>
+      <c r="I12" s="5" t="n"/>
+      <c r="J12" s="9" t="inlineStr">
+        <is>
+          <t>/html/body/div[3]/section[2]/div[2]/ul/li[1]/div/div[1]/div/p|text</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" s="5" t="inlineStr">
+        <is>
+          <t>Business · 스마트 제조</t>
+        </is>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>소분류 링크</t>
+        </is>
+      </c>
+      <c r="D13" s="5" t="inlineStr">
+        <is>
+          <t>문구</t>
+        </is>
+      </c>
+      <c r="E13" s="5" t="n"/>
+      <c r="F13" s="6" t="inlineStr">
+        <is>
+          <t>이차전지 활성화</t>
+        </is>
+      </c>
+      <c r="G13" s="7" t="n"/>
+      <c r="H13" s="8" t="n"/>
+      <c r="I13" s="5" t="inlineStr">
+        <is>
+          <t>사업영역 세부 시트의 소분류 이름과 같은 글 — 한쪽을 바꾸면 함께 고칩니다</t>
+        </is>
+      </c>
+      <c r="J13" s="9" t="inlineStr">
+        <is>
+          <t>/html/body/div[3]/section[2]/div[2]/ul/li[1]/div/div[2]/ul/li[1]/a|text</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" s="5" t="inlineStr">
+        <is>
+          <t>Business · 스마트 제조</t>
+        </is>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>소분류 링크</t>
+        </is>
+      </c>
+      <c r="D14" s="5" t="inlineStr">
+        <is>
+          <t>문구</t>
+        </is>
+      </c>
+      <c r="E14" s="5" t="n"/>
+      <c r="F14" s="6" t="inlineStr">
+        <is>
+          <t>Cycler(Cell&amp;Module)</t>
+        </is>
+      </c>
+      <c r="G14" s="7" t="n"/>
+      <c r="H14" s="8" t="inlineStr">
+        <is>
+          <t>Cycler(Cell&amp;Module)</t>
+        </is>
+      </c>
+      <c r="I14" s="5" t="inlineStr">
+        <is>
+          <t>사업영역 세부 시트의 소분류 이름과 같은 글 — 한쪽을 바꾸면 함께 고칩니다</t>
+        </is>
+      </c>
+      <c r="J14" s="9" t="inlineStr">
+        <is>
+          <t>/html/body/div[3]/section[2]/div[2]/ul/li[1]/div/div[2]/ul/li[2]/a|text</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" s="5" t="inlineStr">
+        <is>
+          <t>Business · 스마트 제조</t>
+        </is>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>소분류 링크</t>
+        </is>
+      </c>
+      <c r="D15" s="5" t="inlineStr">
+        <is>
+          <t>문구</t>
+        </is>
+      </c>
+      <c r="E15" s="5" t="n"/>
+      <c r="F15" s="6" t="inlineStr">
+        <is>
+          <t>자동화 시스템</t>
+        </is>
+      </c>
+      <c r="G15" s="7" t="n"/>
+      <c r="H15" s="8" t="n"/>
+      <c r="I15" s="5" t="inlineStr">
+        <is>
+          <t>사업영역 세부 시트의 소분류 이름과 같은 글 — 한쪽을 바꾸면 함께 고칩니다</t>
+        </is>
+      </c>
+      <c r="J15" s="9" t="inlineStr">
+        <is>
+          <t>/html/body/div[3]/section[2]/div[2]/ul/li[1]/div/div[2]/ul/li[3]/a|text</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" s="5" t="inlineStr">
+        <is>
+          <t>Business · 스마트 제조</t>
+        </is>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>소분류 링크</t>
+        </is>
+      </c>
+      <c r="D16" s="5" t="inlineStr">
+        <is>
+          <t>문구</t>
+        </is>
+      </c>
+      <c r="E16" s="5" t="n"/>
+      <c r="F16" s="6" t="inlineStr">
+        <is>
+          <t>이차전지 소재</t>
+        </is>
+      </c>
+      <c r="G16" s="7" t="n"/>
+      <c r="H16" s="8" t="n"/>
+      <c r="I16" s="5" t="inlineStr">
+        <is>
+          <t>사업영역 세부 시트의 소분류 이름과 같은 글 — 한쪽을 바꾸면 함께 고칩니다</t>
+        </is>
+      </c>
+      <c r="J16" s="9" t="inlineStr">
+        <is>
+          <t>/html/body/div[3]/section[2]/div[2]/ul/li[1]/div/div[2]/ul/li[4]/a|text</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" s="5" t="inlineStr">
+        <is>
+          <t>Business · 에너지 인프라</t>
+        </is>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>카드 설명</t>
+        </is>
+      </c>
+      <c r="D17" s="5" t="inlineStr">
+        <is>
+          <t>문구</t>
+        </is>
+      </c>
+      <c r="E17" s="5" t="n"/>
+      <c r="F17" s="6" t="inlineStr">
+        <is>
+          <t>배터리로 전력을 저장하고, 끊기지 않게 지켜냅니다.
+그리드 규모 ESS부터 우주 발사체 전원까지 아우릅니다.</t>
+        </is>
+      </c>
+      <c r="G17" s="7" t="n"/>
+      <c r="H17" s="8" t="n"/>
+      <c r="I17" s="5" t="n"/>
+      <c r="J17" s="9" t="inlineStr">
+        <is>
+          <t>/html/body/div[3]/section[2]/div[2]/ul/li[2]/div/div[1]/div/p|text</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" s="5" t="inlineStr">
+        <is>
+          <t>Business · 에너지 인프라</t>
+        </is>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>소분류 링크</t>
+        </is>
+      </c>
+      <c r="D18" s="5" t="inlineStr">
+        <is>
+          <t>문구</t>
+        </is>
+      </c>
+      <c r="E18" s="5" t="n"/>
+      <c r="F18" s="6" t="inlineStr">
+        <is>
+          <t>ESS</t>
+        </is>
+      </c>
+      <c r="G18" s="7" t="n"/>
+      <c r="H18" s="8" t="inlineStr">
+        <is>
+          <t>ESS</t>
+        </is>
+      </c>
+      <c r="I18" s="5" t="inlineStr">
+        <is>
+          <t>사업영역 세부 시트의 소분류 이름과 같은 글 — 한쪽을 바꾸면 함께 고칩니다</t>
+        </is>
+      </c>
+      <c r="J18" s="9" t="inlineStr">
+        <is>
+          <t>/html/body/div[3]/section[2]/div[2]/ul/li[2]/div/div[2]/ul/li[1]/a|text</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="5" t="n">
+        <v>18</v>
+      </c>
+      <c r="B19" s="5" t="inlineStr">
+        <is>
+          <t>Business · 에너지 인프라</t>
+        </is>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>소분류 링크</t>
+        </is>
+      </c>
+      <c r="D19" s="5" t="inlineStr">
+        <is>
+          <t>문구</t>
+        </is>
+      </c>
+      <c r="E19" s="5" t="n"/>
+      <c r="F19" s="6" t="inlineStr">
+        <is>
+          <t>UPS</t>
+        </is>
+      </c>
+      <c r="G19" s="7" t="n"/>
+      <c r="H19" s="8" t="inlineStr">
+        <is>
+          <t>UPS</t>
+        </is>
+      </c>
+      <c r="I19" s="5" t="inlineStr">
+        <is>
+          <t>사업영역 세부 시트의 소분류 이름과 같은 글 — 한쪽을 바꾸면 함께 고칩니다</t>
+        </is>
+      </c>
+      <c r="J19" s="9" t="inlineStr">
+        <is>
+          <t>/html/body/div[3]/section[2]/div[2]/ul/li[2]/div/div[2]/ul/li[2]/a|text</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="5" t="n">
+        <v>19</v>
+      </c>
+      <c r="B20" s="5" t="inlineStr">
+        <is>
+          <t>Business · 에너지 인프라</t>
+        </is>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>소분류 링크</t>
+        </is>
+      </c>
+      <c r="D20" s="5" t="inlineStr">
+        <is>
+          <t>문구</t>
+        </is>
+      </c>
+      <c r="E20" s="5" t="n"/>
+      <c r="F20" s="6" t="inlineStr">
+        <is>
+          <t>솔루션</t>
+        </is>
+      </c>
+      <c r="G20" s="7" t="n"/>
+      <c r="H20" s="8" t="n"/>
+      <c r="I20" s="5" t="inlineStr">
+        <is>
+          <t>사업영역 세부 시트의 소분류 이름과 같은 글 — 한쪽을 바꾸면 함께 고칩니다</t>
+        </is>
+      </c>
+      <c r="J20" s="9" t="inlineStr">
+        <is>
+          <t>/html/body/div[3]/section[2]/div[2]/ul/li[2]/div/div[2]/ul/li[3]/a|text</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="5" t="n">
+        <v>20</v>
+      </c>
+      <c r="B21" s="5" t="inlineStr">
+        <is>
+          <t>Business · 인공지능 플랫폼</t>
+        </is>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>카드 설명</t>
+        </is>
+      </c>
+      <c r="D21" s="5" t="inlineStr">
+        <is>
+          <t>문구</t>
+        </is>
+      </c>
+      <c r="E21" s="5" t="n"/>
+      <c r="F21" s="6" t="inlineStr">
+        <is>
+          <t>AI로 배터리와 설비의 상태를 읽어냅니다.
+진단부터 충전·제어까지, 전기 모빌리티의 데이터를 잇습니다.</t>
+        </is>
+      </c>
+      <c r="G21" s="7" t="n"/>
+      <c r="H21" s="8" t="n"/>
+      <c r="I21" s="5" t="n"/>
+      <c r="J21" s="9" t="inlineStr">
+        <is>
+          <t>/html/body/div[3]/section[2]/div[2]/ul/li[3]/div/div[1]/div/p|text</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="5" t="n">
+        <v>21</v>
+      </c>
+      <c r="B22" s="5" t="inlineStr">
+        <is>
+          <t>Business · 인공지능 플랫폼</t>
+        </is>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>소분류 링크</t>
+        </is>
+      </c>
+      <c r="D22" s="5" t="inlineStr">
+        <is>
+          <t>문구</t>
+        </is>
+      </c>
+      <c r="E22" s="5" t="n"/>
+      <c r="F22" s="6" t="inlineStr">
+        <is>
+          <t>로봇 플랫폼</t>
+        </is>
+      </c>
+      <c r="G22" s="7" t="n"/>
+      <c r="H22" s="8" t="n"/>
+      <c r="I22" s="5" t="inlineStr">
+        <is>
+          <t>사업영역 세부 시트의 소분류 이름과 같은 글 — 한쪽을 바꾸면 함께 고칩니다</t>
+        </is>
+      </c>
+      <c r="J22" s="9" t="inlineStr">
+        <is>
+          <t>/html/body/div[3]/section[2]/div[2]/ul/li[3]/div/div[2]/ul/li[1]/a|text</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="5" t="n">
+        <v>22</v>
+      </c>
+      <c r="B23" s="5" t="inlineStr">
+        <is>
+          <t>Business · 인공지능 플랫폼</t>
+        </is>
+      </c>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>소분류 링크</t>
+        </is>
+      </c>
+      <c r="D23" s="5" t="inlineStr">
+        <is>
+          <t>문구</t>
+        </is>
+      </c>
+      <c r="E23" s="5" t="n"/>
+      <c r="F23" s="6" t="inlineStr">
+        <is>
+          <t>배터리 진단 플랫폼</t>
+        </is>
+      </c>
+      <c r="G23" s="7" t="n"/>
+      <c r="H23" s="8" t="n"/>
+      <c r="I23" s="5" t="inlineStr">
+        <is>
+          <t>사업영역 세부 시트의 소분류 이름과 같은 글 — 한쪽을 바꾸면 함께 고칩니다</t>
+        </is>
+      </c>
+      <c r="J23" s="9" t="inlineStr">
+        <is>
+          <t>/html/body/div[3]/section[2]/div[2]/ul/li[3]/div/div[2]/ul/li[2]/a|text</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="5" t="n">
+        <v>23</v>
+      </c>
+      <c r="B24" s="5" t="inlineStr">
+        <is>
+          <t>Business · 인공지능 플랫폼</t>
+        </is>
+      </c>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t>소분류 링크</t>
+        </is>
+      </c>
+      <c r="D24" s="5" t="inlineStr">
+        <is>
+          <t>문구</t>
+        </is>
+      </c>
+      <c r="E24" s="5" t="n"/>
+      <c r="F24" s="6" t="inlineStr">
+        <is>
+          <t>전기자동차 충전 플랫폼</t>
+        </is>
+      </c>
+      <c r="G24" s="7" t="n"/>
+      <c r="H24" s="8" t="n"/>
+      <c r="I24" s="5" t="inlineStr">
+        <is>
+          <t>사업영역 세부 시트의 소분류 이름과 같은 글 — 한쪽을 바꾸면 함께 고칩니다</t>
+        </is>
+      </c>
+      <c r="J24" s="9" t="inlineStr">
+        <is>
+          <t>/html/body/div[3]/section[2]/div[2]/ul/li[3]/div/div[2]/ul/li[3]/a|text</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="5" t="n">
+        <v>24</v>
+      </c>
+      <c r="B25" s="5" t="inlineStr">
+        <is>
+          <t>Business · 인공지능 플랫폼</t>
+        </is>
+      </c>
+      <c r="C25" s="5" t="inlineStr">
+        <is>
+          <t>소분류 링크</t>
+        </is>
+      </c>
+      <c r="D25" s="5" t="inlineStr">
+        <is>
+          <t>문구</t>
+        </is>
+      </c>
+      <c r="E25" s="5" t="n"/>
+      <c r="F25" s="6" t="inlineStr">
+        <is>
+          <t>전기자동차 제어 플랫폼</t>
+        </is>
+      </c>
+      <c r="G25" s="7" t="n"/>
+      <c r="H25" s="8" t="n"/>
+      <c r="I25" s="5" t="inlineStr">
+        <is>
+          <t>사업영역 세부 시트의 소분류 이름과 같은 글 — 한쪽을 바꾸면 함께 고칩니다</t>
+        </is>
+      </c>
+      <c r="J25" s="9" t="inlineStr">
+        <is>
+          <t>/html/body/div[3]/section[2]/div[2]/ul/li[3]/div/div[2]/ul/li[4]/a|text</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="5" t="n">
+        <v>25</v>
+      </c>
+      <c r="B26" s="5" t="inlineStr">
+        <is>
+          <t>Business · 화합물 전력 반도체</t>
+        </is>
+      </c>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t>카드 설명</t>
+        </is>
+      </c>
+      <c r="D26" s="5" t="inlineStr">
+        <is>
+          <t>문구</t>
+        </is>
+      </c>
+      <c r="E26" s="5" t="n"/>
+      <c r="F26" s="6" t="inlineStr">
+        <is>
+          <t>질화갈륨(GaN)을 기반으로 전력반도체와 RF반도체를 설계, 생산합니다.
+국내 최대 규모의 8인치 EPI 양산 체계와 칩 설계 역량을 갖췄습니다</t>
+        </is>
+      </c>
+      <c r="G26" s="7" t="n"/>
+      <c r="H26" s="8" t="n"/>
+      <c r="I26" s="5" t="n"/>
+      <c r="J26" s="9" t="inlineStr">
+        <is>
+          <t>/html/body/div[3]/section[2]/div[2]/ul/li[4]/div/div[1]/div/p|text</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="5" t="n">
+        <v>26</v>
+      </c>
+      <c r="B27" s="5" t="inlineStr">
+        <is>
+          <t>Business · 화합물 전력 반도체</t>
+        </is>
+      </c>
+      <c r="C27" s="5" t="inlineStr">
+        <is>
+          <t>소분류 링크</t>
+        </is>
+      </c>
+      <c r="D27" s="5" t="inlineStr">
+        <is>
+          <t>문구</t>
+        </is>
+      </c>
+      <c r="E27" s="5" t="n"/>
+      <c r="F27" s="6" t="inlineStr">
+        <is>
+          <t>GaN Epi-Wafer</t>
+        </is>
+      </c>
+      <c r="G27" s="7" t="n"/>
+      <c r="H27" s="8" t="inlineStr">
+        <is>
+          <t>GaN Epi-Wafer</t>
+        </is>
+      </c>
+      <c r="I27" s="5" t="inlineStr">
+        <is>
+          <t>사업영역 세부 시트의 소분류 이름과 같은 글 — 한쪽을 바꾸면 함께 고칩니다</t>
+        </is>
+      </c>
+      <c r="J27" s="9" t="inlineStr">
+        <is>
+          <t>/html/body/div[3]/section[2]/div[2]/ul/li[4]/div/div[2]/ul/li[1]/a|text</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="5" t="n">
+        <v>27</v>
+      </c>
+      <c r="B28" s="5" t="inlineStr">
+        <is>
+          <t>Business · 화합물 전력 반도체</t>
+        </is>
+      </c>
+      <c r="C28" s="5" t="inlineStr">
+        <is>
+          <t>소분류 링크</t>
+        </is>
+      </c>
+      <c r="D28" s="5" t="inlineStr">
+        <is>
+          <t>문구</t>
+        </is>
+      </c>
+      <c r="E28" s="5" t="n"/>
+      <c r="F28" s="6" t="inlineStr">
+        <is>
+          <t>GaN Power Device</t>
+        </is>
+      </c>
+      <c r="G28" s="7" t="n"/>
+      <c r="H28" s="8" t="inlineStr">
+        <is>
+          <t>GaN Power Device</t>
+        </is>
+      </c>
+      <c r="I28" s="5" t="inlineStr">
+        <is>
+          <t>사업영역 세부 시트의 소분류 이름과 같은 글 — 한쪽을 바꾸면 함께 고칩니다</t>
+        </is>
+      </c>
+      <c r="J28" s="9" t="inlineStr">
+        <is>
+          <t>/html/body/div[3]/section[2]/div[2]/ul/li[4]/div/div[2]/ul/li[2]/a|text</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="5" t="n">
+        <v>28</v>
+      </c>
+      <c r="B29" s="5" t="inlineStr">
+        <is>
+          <t>Business · 화합물 전력 반도체</t>
+        </is>
+      </c>
+      <c r="C29" s="5" t="inlineStr">
+        <is>
+          <t>소분류 링크</t>
+        </is>
+      </c>
+      <c r="D29" s="5" t="inlineStr">
+        <is>
+          <t>문구</t>
+        </is>
+      </c>
+      <c r="E29" s="5" t="n"/>
+      <c r="F29" s="6" t="inlineStr">
+        <is>
+          <t>에이프로 세미콘</t>
+        </is>
+      </c>
+      <c r="G29" s="7" t="n"/>
+      <c r="H29" s="8" t="n"/>
+      <c r="I29" s="5" t="inlineStr">
+        <is>
+          <t>사업영역 세부 시트의 소분류 이름과 같은 글 — 한쪽을 바꾸면 함께 고칩니다</t>
+        </is>
+      </c>
+      <c r="J29" s="9" t="inlineStr">
+        <is>
+          <t>/html/body/div[3]/section[2]/div[2]/ul/li[4]/div/div[2]/ul/li[3]/a|text</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="5" t="n">
+        <v>29</v>
+      </c>
+      <c r="B30" s="5" t="inlineStr">
+        <is>
+          <t>Who we are</t>
+        </is>
+      </c>
+      <c r="C30" s="5" t="inlineStr">
+        <is>
+          <t>섹션 제목</t>
+        </is>
+      </c>
+      <c r="D30" s="5" t="inlineStr">
+        <is>
+          <t>문구</t>
+        </is>
+      </c>
+      <c r="E30" s="5" t="n"/>
+      <c r="F30" s="6" t="inlineStr">
+        <is>
+          <t>Who we are</t>
+        </is>
+      </c>
+      <c r="G30" s="7" t="n"/>
+      <c r="H30" s="8" t="inlineStr">
+        <is>
+          <t>Who we are</t>
+        </is>
+      </c>
+      <c r="I30" s="5" t="n"/>
+      <c r="J30" s="9" t="inlineStr">
+        <is>
+          <t>/html/body/div[3]/section[3]/h2|text</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="5" t="n">
+        <v>30</v>
+      </c>
+      <c r="B31" s="5" t="inlineStr">
+        <is>
+          <t>Who we are</t>
+        </is>
+      </c>
+      <c r="C31" s="5" t="inlineStr">
+        <is>
+          <t>섹션 라벨</t>
+        </is>
+      </c>
+      <c r="D31" s="5" t="inlineStr">
+        <is>
+          <t>문구</t>
+        </is>
+      </c>
+      <c r="E31" s="5" t="n"/>
+      <c r="F31" s="6" t="inlineStr">
+        <is>
+          <t>핵심역량</t>
+        </is>
+      </c>
+      <c r="G31" s="7" t="n"/>
+      <c r="H31" s="8" t="n"/>
+      <c r="I31" s="5" t="n"/>
+      <c r="J31" s="9" t="inlineStr">
+        <is>
+          <t>/html/body/div[3]/section[3]/h2/span|text</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="5" t="n">
+        <v>31</v>
+      </c>
+      <c r="B32" s="5" t="inlineStr">
+        <is>
+          <t>Who we are · 01</t>
+        </is>
+      </c>
+      <c r="C32" s="5" t="inlineStr">
+        <is>
+          <t>번호</t>
+        </is>
+      </c>
+      <c r="D32" s="5" t="inlineStr">
+        <is>
+          <t>번호</t>
+        </is>
+      </c>
+      <c r="E32" s="5" t="n"/>
+      <c r="F32" s="6" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="G32" s="6" t="n"/>
+      <c r="H32" s="6" t="n"/>
+      <c r="I32" s="5" t="n"/>
+      <c r="J32" s="9" t="inlineStr">
+        <is>
+          <t>/html/body/div[3]/section[3]/ol/li[1]/div/div/div/div/span|text</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="5" t="n">
+        <v>32</v>
+      </c>
+      <c r="B33" s="5" t="inlineStr">
+        <is>
+          <t>Who we are · 01</t>
+        </is>
+      </c>
+      <c r="C33" s="5" t="inlineStr">
+        <is>
+          <t>제목</t>
+        </is>
+      </c>
+      <c r="D33" s="5" t="inlineStr">
+        <is>
+          <t>문구</t>
+        </is>
+      </c>
+      <c r="E33" s="5" t="n"/>
+      <c r="F33" s="6" t="inlineStr">
+        <is>
+          <t>전력 변환 기술 기반의 Total Energy Solution</t>
+        </is>
+      </c>
+      <c r="G33" s="7" t="n"/>
+      <c r="H33" s="8" t="n"/>
+      <c r="I33" s="5" t="n"/>
+      <c r="J33" s="9" t="inlineStr">
+        <is>
+          <t>/html/body/div[3]/section[3]/ol/li[1]/div/div/div/div/h3|text</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="5" t="n">
+        <v>33</v>
+      </c>
+      <c r="B34" s="5" t="inlineStr">
+        <is>
+          <t>Who we are · 01</t>
+        </is>
+      </c>
+      <c r="C34" s="5" t="inlineStr">
+        <is>
+          <t>문단</t>
+        </is>
+      </c>
+      <c r="D34" s="5" t="inlineStr">
+        <is>
+          <t>문구</t>
+        </is>
+      </c>
+      <c r="E34" s="5" t="n"/>
+      <c r="F34" s="6" t="inlineStr">
+        <is>
+          <t>에이프로는 2차전지 활성화 공정 장비부터 ESS, 초고속 전기차 충전 인프라, 우주 발사체 전원 시스템까지 폭넓은 포트폴리오를 구축하고 있습니다. 끊임없는 연구개발을 통해 고효율, 고밀도 전력 변환 기술을 고도화하며 지속 가능한 미래 에너지 생태계를 완성해 나갑니다.</t>
+        </is>
+      </c>
+      <c r="G34" s="7" t="n"/>
+      <c r="H34" s="8" t="n"/>
+      <c r="I34" s="5" t="n"/>
+      <c r="J34" s="9" t="inlineStr">
+        <is>
+          <t>/html/body/div[3]/section[3]/ol/li[1]/div/div/div/p|text</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="5" t="n">
+        <v>34</v>
+      </c>
+      <c r="B35" s="5" t="inlineStr">
+        <is>
+          <t>Who we are · 02</t>
+        </is>
+      </c>
+      <c r="C35" s="5" t="inlineStr">
+        <is>
+          <t>번호</t>
+        </is>
+      </c>
+      <c r="D35" s="5" t="inlineStr">
+        <is>
+          <t>번호</t>
+        </is>
+      </c>
+      <c r="E35" s="5" t="n"/>
+      <c r="F35" s="6" t="inlineStr">
+        <is>
+          <t>02</t>
+        </is>
+      </c>
+      <c r="G35" s="6" t="n"/>
+      <c r="H35" s="6" t="n"/>
+      <c r="I35" s="5" t="n"/>
+      <c r="J35" s="9" t="inlineStr">
+        <is>
+          <t>/html/body/div[3]/section[3]/ol/li[2]/div/div/div/div/span|text</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="5" t="n">
+        <v>35</v>
+      </c>
+      <c r="B36" s="5" t="inlineStr">
+        <is>
+          <t>Who we are · 02</t>
+        </is>
+      </c>
+      <c r="C36" s="5" t="inlineStr">
+        <is>
+          <t>제목</t>
+        </is>
+      </c>
+      <c r="D36" s="5" t="inlineStr">
+        <is>
+          <t>문구</t>
+        </is>
+      </c>
+      <c r="E36" s="5" t="n"/>
+      <c r="F36" s="6" t="inlineStr">
+        <is>
+          <t>소재부터 시스템까지 잇는 수직 계열화 역량 (Materials to System)</t>
+        </is>
+      </c>
+      <c r="G36" s="7" t="n"/>
+      <c r="H36" s="8" t="n"/>
+      <c r="I36" s="5" t="n"/>
+      <c r="J36" s="9" t="inlineStr">
+        <is>
+          <t>/html/body/div[3]/section[3]/ol/li[2]/div/div/div/div/h3|text</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="5" t="n">
+        <v>36</v>
+      </c>
+      <c r="B37" s="5" t="inlineStr">
+        <is>
+          <t>Who we are · 02</t>
+        </is>
+      </c>
+      <c r="C37" s="5" t="inlineStr">
+        <is>
+          <t>문단</t>
+        </is>
+      </c>
+      <c r="D37" s="5" t="inlineStr">
+        <is>
+          <t>문구</t>
+        </is>
+      </c>
+      <c r="E37" s="5" t="n"/>
+      <c r="F37" s="6" t="inlineStr">
+        <is>
+          <t>우리의 혁신은 시스템의 가장 깊은 곳, '반도체'에서 시작됩니다. 차세대 고효율 질화갈륨(GaN) 전력반도체 핵심 소재(Epi-Wafer)와 소자를 직접 설계하고 내재화함으로써, 기존의 한계를 뛰어넘는 초소형·초고효율 전력 변환 모듈을 실현합니다.</t>
+        </is>
+      </c>
+      <c r="G37" s="7" t="n"/>
+      <c r="H37" s="8" t="n"/>
+      <c r="I37" s="5" t="n"/>
+      <c r="J37" s="9" t="inlineStr">
+        <is>
+          <t>/html/body/div[3]/section[3]/ol/li[2]/div/div/div/p|text</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="5" t="n">
+        <v>37</v>
+      </c>
+      <c r="B38" s="5" t="inlineStr">
+        <is>
+          <t>Who we are · 03</t>
+        </is>
+      </c>
+      <c r="C38" s="5" t="inlineStr">
+        <is>
+          <t>번호</t>
+        </is>
+      </c>
+      <c r="D38" s="5" t="inlineStr">
+        <is>
+          <t>번호</t>
+        </is>
+      </c>
+      <c r="E38" s="5" t="n"/>
+      <c r="F38" s="6" t="inlineStr">
+        <is>
+          <t>03</t>
+        </is>
+      </c>
+      <c r="G38" s="6" t="n"/>
+      <c r="H38" s="6" t="n"/>
+      <c r="I38" s="5" t="n"/>
+      <c r="J38" s="9" t="inlineStr">
+        <is>
+          <t>/html/body/div[3]/section[3]/ol/li[3]/div/div/div/div/span|text</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="5" t="n">
+        <v>38</v>
+      </c>
+      <c r="B39" s="5" t="inlineStr">
+        <is>
+          <t>Who we are · 03</t>
+        </is>
+      </c>
+      <c r="C39" s="5" t="inlineStr">
+        <is>
+          <t>제목</t>
+        </is>
+      </c>
+      <c r="D39" s="5" t="inlineStr">
+        <is>
+          <t>문구</t>
+        </is>
+      </c>
+      <c r="E39" s="5" t="n"/>
+      <c r="F39" s="6" t="inlineStr">
+        <is>
+          <t>In-house 설계를 통한 완벽한 시스템 통합 (SI) 및 지능형 플랫폼</t>
+        </is>
+      </c>
+      <c r="G39" s="7" t="n"/>
+      <c r="H39" s="8" t="n"/>
+      <c r="I39" s="5" t="n"/>
+      <c r="J39" s="9" t="inlineStr">
+        <is>
+          <t>/html/body/div[3]/section[3]/ol/li[3]/div/div/div/div/h3|text</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="5" t="n">
+        <v>39</v>
+      </c>
+      <c r="B40" s="5" t="inlineStr">
+        <is>
+          <t>Who we are · 03</t>
+        </is>
+      </c>
+      <c r="C40" s="5" t="inlineStr">
+        <is>
+          <t>문단</t>
+        </is>
+      </c>
+      <c r="D40" s="5" t="inlineStr">
+        <is>
+          <t>문구</t>
+        </is>
+      </c>
+      <c r="E40" s="5" t="n"/>
+      <c r="F40" s="6" t="inlineStr">
+        <is>
+          <t>기구, 회로, 소프트웨어에 이르는 100% In-house 설계 역량을 통해 고객의 다양한 요구에 최적화된 하드웨어 시스템을 구축합니다. 나아가 AI 기반의 배터리 진단 플랫폼과 산업 안전 로보틱스 등 지능형 소프트웨어를 융합하여, 시스템의 안정성과 운영 효율을 극대화하는 스마트 솔루션을 제공합니다.</t>
+        </is>
+      </c>
+      <c r="G40" s="7" t="n"/>
+      <c r="H40" s="8" t="n"/>
+      <c r="I40" s="5" t="n"/>
+      <c r="J40" s="9" t="inlineStr">
+        <is>
+          <t>/html/body/div[3]/section[3]/ol/li[3]/div/div/div/p|text</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="5" t="n">
+        <v>40</v>
+      </c>
+      <c r="B41" s="5" t="inlineStr">
+        <is>
+          <t>Who we are · 04</t>
+        </is>
+      </c>
+      <c r="C41" s="5" t="inlineStr">
+        <is>
+          <t>번호</t>
+        </is>
+      </c>
+      <c r="D41" s="5" t="inlineStr">
+        <is>
+          <t>번호</t>
+        </is>
+      </c>
+      <c r="E41" s="5" t="n"/>
+      <c r="F41" s="6" t="inlineStr">
+        <is>
+          <t>04</t>
+        </is>
+      </c>
+      <c r="G41" s="6" t="n"/>
+      <c r="H41" s="6" t="n"/>
+      <c r="I41" s="5" t="n"/>
+      <c r="J41" s="9" t="inlineStr">
+        <is>
+          <t>/html/body/div[3]/section[3]/ol/li[4]/div/div/div/div/span|text</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="5" t="n">
+        <v>41</v>
+      </c>
+      <c r="B42" s="5" t="inlineStr">
+        <is>
+          <t>Who we are · 04</t>
+        </is>
+      </c>
+      <c r="C42" s="5" t="inlineStr">
+        <is>
+          <t>제목</t>
+        </is>
+      </c>
+      <c r="D42" s="5" t="inlineStr">
+        <is>
+          <t>문구</t>
+        </is>
+      </c>
+      <c r="E42" s="5" t="n"/>
+      <c r="F42" s="6" t="inlineStr">
+        <is>
+          <t>세계를 무대로 하는 글로벌 파트너</t>
+        </is>
+      </c>
+      <c r="G42" s="7" t="n"/>
+      <c r="H42" s="8" t="n"/>
+      <c r="I42" s="5" t="n"/>
+      <c r="J42" s="9" t="inlineStr">
+        <is>
+          <t>/html/body/div[3]/section[3]/ol/li[4]/div/div/div/div/h3|text</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="5" t="n">
+        <v>42</v>
+      </c>
+      <c r="B43" s="5" t="inlineStr">
+        <is>
+          <t>Who we are · 04</t>
+        </is>
+      </c>
+      <c r="C43" s="5" t="inlineStr">
+        <is>
+          <t>문단</t>
+        </is>
+      </c>
+      <c r="D43" s="5" t="inlineStr">
+        <is>
+          <t>문구</t>
+        </is>
+      </c>
+      <c r="E43" s="5" t="n"/>
+      <c r="F43" s="6" t="inlineStr">
+        <is>
+          <t>미국, 유럽, 중국, 동남아시아 등 전 세계 핵심 거점에 현지 법인과 전문가 네트워크를 구축했습니다. 글로벌 탑티어 배터리 제조사 및 완성차 기업들과 긴밀히 협력하며, 어떤 환경에서도 기민(Agile)하게 대응하고 최고 품질의 고객 지원을 약속합니다.</t>
+        </is>
+      </c>
+      <c r="G43" s="7" t="n"/>
+      <c r="H43" s="8" t="n"/>
+      <c r="I43" s="5" t="n"/>
+      <c r="J43" s="9" t="inlineStr">
+        <is>
+          <t>/html/body/div[3]/section[3]/ol/li[4]/div/div/div/p|text</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="5" t="n">
+        <v>43</v>
+      </c>
+      <c r="B44" s="5" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="C44" s="5" t="inlineStr">
+        <is>
+          <t>섹션 제목</t>
+        </is>
+      </c>
+      <c r="D44" s="5" t="inlineStr">
+        <is>
+          <t>문구</t>
+        </is>
+      </c>
+      <c r="E44" s="5" t="n"/>
+      <c r="F44" s="6" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="G44" s="7" t="n"/>
+      <c r="H44" s="8" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="I44" s="5" t="n"/>
+      <c r="J44" s="9" t="inlineStr">
+        <is>
+          <t>/html/body/div[3]/section[4]/div[1]/div/h2|text</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="5" t="n">
+        <v>44</v>
+      </c>
+      <c r="B45" s="5" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="C45" s="5" t="inlineStr">
+        <is>
+          <t>섹션 라벨</t>
+        </is>
+      </c>
+      <c r="D45" s="5" t="inlineStr">
+        <is>
+          <t>문구</t>
+        </is>
+      </c>
+      <c r="E45" s="5" t="n"/>
+      <c r="F45" s="6" t="inlineStr">
+        <is>
+          <t>보도자료</t>
+        </is>
+      </c>
+      <c r="G45" s="7" t="n"/>
+      <c r="H45" s="8" t="n"/>
+      <c r="I45" s="5" t="n"/>
+      <c r="J45" s="9" t="inlineStr">
+        <is>
+          <t>/html/body/div[3]/section[4]/div[1]/div/h2/span|text</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="5" t="n">
+        <v>45</v>
+      </c>
+      <c r="B46" s="5" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="C46" s="5" t="inlineStr">
+        <is>
+          <t>더보기 단추</t>
+        </is>
+      </c>
+      <c r="D46" s="5" t="inlineStr">
+        <is>
+          <t>문구</t>
+        </is>
+      </c>
+      <c r="E46" s="5" t="n"/>
+      <c r="F46" s="6" t="inlineStr">
+        <is>
+          <t>더보기</t>
+        </is>
+      </c>
+      <c r="G46" s="7" t="n"/>
+      <c r="H46" s="8" t="n"/>
+      <c r="I46" s="5" t="n"/>
+      <c r="J46" s="9" t="inlineStr">
+        <is>
+          <t>/html/body/div[3]/section[4]/div[1]/a|text</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="5" t="n">
+        <v>46</v>
+      </c>
+      <c r="B47" s="5" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="C47" s="5" t="inlineStr">
+        <is>
+          <t>목록 '자세히 보기'</t>
+        </is>
+      </c>
+      <c r="D47" s="5" t="inlineStr">
+        <is>
+          <t>문구</t>
+        </is>
+      </c>
+      <c r="E47" s="5" t="n"/>
+      <c r="F47" s="6" t="inlineStr">
+        <is>
+          <t>자세히 보기</t>
+        </is>
+      </c>
+      <c r="G47" s="7" t="n"/>
+      <c r="H47" s="8" t="n"/>
+      <c r="I47" s="5" t="inlineStr">
+        <is>
+          <t>같은 문구 5 곳 — 한 줄로 합침</t>
+        </is>
+      </c>
+      <c r="J47" s="9" t="inlineStr">
+        <is>
+          <t>/html/body/div[3]/section[4]/ul/li[1]/a/span[3]/span|text
+/html/body/div[3]/section[4]/ul/li[2]/a/span[3]/span|text
+/html/body/div[3]/section[4]/ul/li[3]/a/span[3]/span|text
+/html/body/div[3]/section[4]/ul/li[4]/a/span[3]/span|text
+/html/body/div[3]/section[4]/ul/li[5]/a/span[3]/span|text</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:J47"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -5839,7 +7651,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -12737,7 +14549,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -14541,7 +16353,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>